<commit_message>
test(fm): add insurance_conditions units sc23/sc24 for IL ordering (#2040)
sc23 reproduces issue #2040: one location under a single condition covered by
three policy-layers where two share condition terms and one differs. Before the
cond-all layer-preservation fix this collapses order-dependently, so loss_il
changes when account.csv rows are reordered; the regenerated expected output
fails on unfixed main and passes with the fix.

sc24 is the edge case: three co-insurance layers on one condition with identical
condition terms differing only in LayerParticipation. Those layers collapse
harmlessly, guarding that the fix stays a no-op when all layers share a profile.

Includes the regenerated combined CSVs, expected/ and expected_subperils/
outputs, units.txt registration, and the test-case list workbook row.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/validation/insurance_conditions_test_case_list.xlsx
+++ b/validation/insurance_conditions_test_case_list.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="24.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1307,6 +1307,78 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>sc23</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Issue #2040: one location under a single condition covered by three policy-layers; two share condition terms and one differs. Reproduces account-row-order dependence of loss_il (order-dependent before the cond-all layer-preservation fix).</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>sc24</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Edge case: three co-insurance policy-layers on one condition with identical condition terms, differing only in LayerParticipation. Layers collapse harmlessly; guards that the fix stays a no-op when all layers share a profile.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>